<commit_message>
Put back the spaces the PDF extraction dropped in risk text
pdfplumber's default 3 pt word gap glued words in the book's narrow justified
cells ("Kesugihandengan", "JangkaMenengah"); at 1.5 pt it separates them but
also splits words the PDF letter-spaced ("pemeliha raan"). Neither read is
the book.

respace_risk_text.py reads each fixture's own table at both gaps and adds a
space only where every piece left is a word the book uses standing alone (or
a number, unit, acronym, or a lower->Upper join). It never changes a letter,
so reviewed and hand-edited cells can only gain spaces. 536 cells in 24
fixtures; 101 joins with no safe split are left and listed.

risk_rows takes an x_tolerance; the section -> fixture map moves from the
count test into _kerawanan_sections so both use one list.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/ss_bdgsel_nubrg_ingest.xlsx
+++ b/samples/ss_bdgsel_nubrg_ingest.xlsx
@@ -709,25 +709,16 @@
           <t>500 kV</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -784,15 +775,11 @@
       <c r="J3" t="n">
         <v>1</v>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
           <t>Rawan</t>
@@ -859,15 +846,11 @@
       <c r="J4" t="n">
         <v>1</v>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
           <t>Rawan</t>
@@ -916,25 +899,16 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -973,25 +947,16 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -1030,19 +995,11 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
           <t>Rawan</t>
@@ -1091,25 +1048,16 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -1148,19 +1096,11 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
           <t>Rawan</t>
@@ -1209,29 +1149,21 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>bus section + kopel</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -1270,25 +1202,16 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -1327,25 +1250,16 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -1384,25 +1298,16 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -1441,19 +1346,11 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
           <t>Rawan</t>
@@ -1502,19 +1399,11 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
           <t>Rawan</t>
@@ -1563,25 +1452,16 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -1620,25 +1500,16 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -1695,25 +1566,21 @@
       <c r="J18" t="n">
         <v>2</v>
       </c>
-      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>IBT 150/70 kV</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -1752,25 +1619,16 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -1809,25 +1667,16 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -1866,25 +1715,16 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -1923,19 +1763,11 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
           <t>Rawan</t>
@@ -1984,25 +1816,16 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -2041,25 +1864,16 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -2098,25 +1912,16 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -2155,25 +1960,16 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -2212,25 +2008,16 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -2269,25 +2056,16 @@
           <t>500 kV</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -2344,15 +2122,11 @@
       <c r="J29" t="n">
         <v>1</v>
       </c>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
         <is>
           <t>Rawan</t>
@@ -2419,15 +2193,11 @@
       <c r="J30" t="n">
         <v>1</v>
       </c>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr">
         <is>
           <t>Rawan</t>
@@ -2476,25 +2246,16 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -2533,25 +2294,16 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -2590,25 +2342,16 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -2647,19 +2390,11 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
         <is>
           <t>Rawan</t>
@@ -2708,25 +2443,16 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -2765,25 +2491,16 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -2822,25 +2539,16 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -2879,19 +2587,11 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr">
         <is>
           <t>Rawan</t>
@@ -2940,25 +2640,16 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -2997,25 +2688,16 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -3054,25 +2736,16 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -3111,25 +2784,16 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -3168,25 +2832,16 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -3225,25 +2880,16 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q44" t="inlineStr"/>
       <c r="R44" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -3282,19 +2928,11 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr">
         <is>
           <t>Rawan</t>
@@ -3343,29 +2981,21 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
           <t>bus section + kopel</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -3404,23 +3034,16 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
           <t>bus section + kopel</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr">
         <is>
           <t>Rawan</t>
@@ -3487,25 +3110,21 @@
       <c r="J48" t="n">
         <v>2</v>
       </c>
-      <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
           <t>IBT 150/70 kV</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -3544,25 +3163,16 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr">
         <is>
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q49" t="inlineStr"/>
       <c r="R49" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -3601,17 +3211,11 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
           <t>batas ke Subsistem Pelabuhan Ratu</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr">
         <is>
           <t>Beroperasi</t>
@@ -3627,7 +3231,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -3666,17 +3269,11 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
           <t>batas ke Subsistem Pelabuhan Ratu</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr">
         <is>
           <t>Beroperasi</t>
@@ -3692,7 +3289,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q51" t="inlineStr"/>
       <c r="R51" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -3731,17 +3327,11 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
           <t>batas ke UP2B Jakarta &amp; Banten</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr">
         <is>
           <t>Beroperasi</t>
@@ -3757,7 +3347,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q52" t="inlineStr"/>
       <c r="R52" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -3796,17 +3385,11 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
           <t>batas ke Subsistem Cirata 1,2,3</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr">
         <is>
           <t>Beroperasi</t>
@@ -3822,7 +3405,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q53" t="inlineStr"/>
       <c r="R53" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -3861,17 +3443,11 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
           <t>batas ke Subsistem Cirata 1,2,3</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr">
         <is>
           <t>Beroperasi</t>
@@ -3930,17 +3506,11 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
           <t>penyulang traksi</t>
         </is>
       </c>
-      <c r="M55" t="inlineStr"/>
       <c r="N55" t="inlineStr">
         <is>
           <t>Beroperasi</t>
@@ -3956,7 +3526,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q55" t="inlineStr"/>
       <c r="R55" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -3995,17 +3564,11 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
           <t>batas ke Subsistem Tasikmalaya 1,2</t>
         </is>
       </c>
-      <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr">
         <is>
           <t>Beroperasi</t>
@@ -4021,7 +3584,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q56" t="inlineStr"/>
       <c r="R56" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -4060,17 +3622,11 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
           <t>batas ke Subsistem Mandirancan 1,2</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr"/>
       <c r="N57" t="inlineStr">
         <is>
           <t>Beroperasi</t>
@@ -4086,7 +3642,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q57" t="inlineStr"/>
       <c r="R57" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -4125,17 +3680,11 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
           <t>batas ke Subsistem Mandirancan 1,2</t>
         </is>
       </c>
-      <c r="M58" t="inlineStr"/>
       <c r="N58" t="inlineStr">
         <is>
           <t>Beroperasi</t>
@@ -4151,7 +3700,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q58" t="inlineStr"/>
       <c r="R58" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -4190,17 +3738,11 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
           <t>batas ke Subsistem Mandirancan 1,2</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr"/>
       <c r="N59" t="inlineStr">
         <is>
           <t>Beroperasi</t>
@@ -4216,7 +3758,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q59" t="inlineStr"/>
       <c r="R59" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -4255,17 +3796,11 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
           <t>batas ke sisi Bandung Selatan</t>
         </is>
       </c>
-      <c r="M60" t="inlineStr"/>
       <c r="N60" t="inlineStr">
         <is>
           <t>Beroperasi</t>
@@ -4281,7 +3816,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q60" t="inlineStr"/>
       <c r="R60" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -4320,17 +3854,11 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
           <t>batas ke sisi Bandung Selatan</t>
         </is>
       </c>
-      <c r="M61" t="inlineStr"/>
       <c r="N61" t="inlineStr">
         <is>
           <t>Beroperasi</t>
@@ -4346,7 +3874,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q61" t="inlineStr"/>
       <c r="R61" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -4463,7 +3990,6 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>Outlet PLTA Rajamandala</t>
@@ -4484,7 +4010,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
         <v>1</v>
       </c>
@@ -4498,8 +4023,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -4526,7 +4049,6 @@
       <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>Outlet PLTP Wayang Windu</t>
@@ -4547,7 +4069,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
         <v>1</v>
       </c>
@@ -4561,8 +4082,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -4614,7 +4133,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
         <v>2</v>
       </c>
@@ -4628,8 +4146,6 @@
           <t>Sangat Rawan</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -4656,7 +4172,6 @@
       <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>SUTT Bandung Selatan - Cigereleng</t>
@@ -4677,7 +4192,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
         <v>2</v>
       </c>
@@ -4691,8 +4205,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -4719,7 +4231,6 @@
       <c r="A6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>SUTT Bandung Selatan - Dayeuh Kolot</t>
@@ -4740,7 +4251,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
         <v>2</v>
       </c>
@@ -4754,8 +4264,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -4782,7 +4290,6 @@
       <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>SUTT Bandung Selatan - Panasia</t>
@@ -4803,7 +4310,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
         <v>2</v>
       </c>
@@ -4817,8 +4323,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -4870,7 +4374,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>2</v>
       </c>
@@ -4884,8 +4387,6 @@
           <t>Sangat Rawan</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -4937,7 +4438,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
         <v>2</v>
       </c>
@@ -4951,8 +4451,6 @@
           <t>Sangat Rawan</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -5004,7 +4502,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
         <v>2</v>
       </c>
@@ -5018,8 +4515,6 @@
           <t>Sangat Rawan</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -5046,7 +4541,6 @@
       <c r="A11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>SUTT Sukaluyu - Lengkong Dar (arah SS Cirata)</t>
@@ -5067,7 +4561,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
         <v>2</v>
       </c>
@@ -5081,8 +4574,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -5109,7 +4600,6 @@
       <c r="A12" t="n">
         <v>11</v>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>SUTT Cigereleng - Cibereum</t>
@@ -5130,7 +4620,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
         <v>2</v>
       </c>
@@ -5144,8 +4633,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -5172,7 +4659,6 @@
       <c r="A13" t="n">
         <v>12</v>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>SUTT Cigereleng - Braga</t>
@@ -5193,7 +4679,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
         <v>2</v>
       </c>
@@ -5207,8 +4692,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -5235,7 +4718,6 @@
       <c r="A14" t="n">
         <v>13</v>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>SUTT Cianjur - Lembur Situ (arah UP2B Jakban)</t>
@@ -5256,7 +4738,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
         <v>2</v>
       </c>
@@ -5270,8 +4751,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -5298,7 +4777,6 @@
       <c r="A15" t="n">
         <v>14</v>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>SUTT Cianjur - Bogor Baru (arah UP2B Jakban)</t>
@@ -5319,7 +4797,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
         <v>2</v>
       </c>
@@ -5333,8 +4810,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -5361,7 +4836,6 @@
       <c r="A16" t="n">
         <v>15</v>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
           <t>SUTT Cianjur - Tajur (arah UP2B Jakban)</t>
@@ -5382,7 +4856,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
         <v>2</v>
       </c>
@@ -5396,8 +4869,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -5424,7 +4895,6 @@
       <c r="A17" t="n">
         <v>16</v>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
           <t>SUTT 70 kV Cigereleng - Cikalong</t>
@@ -5445,7 +4915,6 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
         <v>1</v>
       </c>
@@ -5459,8 +4928,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -5487,7 +4954,6 @@
       <c r="A18" t="n">
         <v>17</v>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>SUTT 70 kV Cigereleng - Lamajan</t>
@@ -5508,7 +4974,6 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
         <v>1</v>
       </c>
@@ -5522,8 +4987,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -5575,7 +5038,6 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
         <v>1</v>
       </c>
@@ -5589,8 +5051,6 @@
           <t>Sangat Rawan</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -5617,7 +5077,6 @@
       <c r="A20" t="n">
         <v>19</v>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>SUTT 70 kV Cigereleng - Majalaya</t>
@@ -5638,7 +5097,6 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
         <v>1</v>
       </c>
@@ -5652,8 +5110,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -5680,7 +5136,6 @@
       <c r="A21" t="n">
         <v>20</v>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>SUTT 70 kV Majalaya - Plengan</t>
@@ -5701,7 +5156,6 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
         <v>2</v>
       </c>
@@ -5715,8 +5169,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -5743,7 +5195,6 @@
       <c r="A22" t="n">
         <v>21</v>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>Outlet PLTA Plengan</t>
@@ -5764,7 +5215,6 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
         <v>1</v>
       </c>
@@ -5778,8 +5228,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -5806,7 +5254,6 @@
       <c r="A23" t="n">
         <v>22</v>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>SUTT 70 kV Sumedang Raya - Pameungpeuk</t>
@@ -5827,7 +5274,6 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
         <v>2</v>
       </c>
@@ -5841,8 +5287,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -5869,7 +5313,6 @@
       <c r="A24" t="n">
         <v>23</v>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>SUTT 70 kV Sentosa - Sumedang Raya</t>
@@ -5890,7 +5333,6 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
         <v>2</v>
       </c>
@@ -5904,8 +5346,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -5932,7 +5372,6 @@
       <c r="A25" t="n">
         <v>24</v>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
           <t>Outlet PLTP Kamojang</t>
@@ -5953,7 +5392,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
         <v>1</v>
       </c>
@@ -5967,8 +5405,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -5995,7 +5431,6 @@
       <c r="A26" t="n">
         <v>25</v>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
           <t>Outlet PLTP Darajat</t>
@@ -6016,7 +5451,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
         <v>1</v>
       </c>
@@ -6030,8 +5464,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -6058,7 +5490,6 @@
       <c r="A27" t="n">
         <v>26</v>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
           <t>Outlet PLTA Jatigede</t>
@@ -6079,7 +5510,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
         <v>1</v>
       </c>
@@ -6093,8 +5523,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -6121,7 +5549,6 @@
       <c r="A28" t="n">
         <v>27</v>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
           <t>SUTT Kamojang - Wayang Windu (arah sisi Bandung Selatan)</t>
@@ -6142,7 +5569,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
         <v>2</v>
       </c>
@@ -6156,8 +5582,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -6209,7 +5633,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
         <v>2</v>
       </c>
@@ -6223,8 +5646,6 @@
           <t>Sangat Rawan</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -6251,7 +5672,6 @@
       <c r="A30" t="n">
         <v>29</v>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
           <t>SUTT Darajat - Garut (arah SS Tasikmalaya)</t>
@@ -6272,7 +5692,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
         <v>2</v>
       </c>
@@ -6286,8 +5705,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -6314,7 +5731,6 @@
       <c r="A31" t="n">
         <v>30</v>
       </c>
-      <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
           <t>SUTT Darajat - Rancaekek</t>
@@ -6335,7 +5751,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
         <v>2</v>
       </c>
@@ -6349,8 +5764,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -6402,7 +5815,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
         <v>2</v>
       </c>
@@ -6416,8 +5828,6 @@
           <t>Sangat Rawan</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -6444,7 +5854,6 @@
       <c r="A33" t="n">
         <v>32</v>
       </c>
-      <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
           <t>SUTT Jatigede - Seragi (arah SS Mandirancan)</t>
@@ -6465,7 +5874,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
         <v>2</v>
       </c>
@@ -6479,8 +5887,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -6507,7 +5913,6 @@
       <c r="A34" t="n">
         <v>33</v>
       </c>
-      <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
           <t>SUTT Jatigede - New Kadipaten (arah SS Mandirancan)</t>
@@ -6528,7 +5933,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
         <v>2</v>
       </c>
@@ -6542,8 +5946,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -6570,7 +5972,6 @@
       <c r="A35" t="n">
         <v>34</v>
       </c>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
           <t>SUTT New Ujungberung - Nanjung Rancaekek Baru</t>
@@ -6591,7 +5992,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
         <v>2</v>
       </c>
@@ -6605,8 +6005,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -6633,7 +6031,6 @@
       <c r="A36" t="n">
         <v>35</v>
       </c>
-      <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
           <t>SUTT New Ujungberung - Ujung Berung</t>
@@ -6654,7 +6051,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
         <v>2</v>
       </c>
@@ -6668,8 +6064,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -6696,7 +6090,6 @@
       <c r="A37" t="n">
         <v>36</v>
       </c>
-      <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
           <t>SUTT Cikasungka - Rancaekek Baru</t>
@@ -6717,7 +6110,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
         <v>2</v>
       </c>
@@ -6731,8 +6123,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -6759,7 +6149,6 @@
       <c r="A38" t="n">
         <v>37</v>
       </c>
-      <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
           <t>SUTT Rancaekek - Rancaekek Baru</t>
@@ -6780,7 +6169,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
         <v>2</v>
       </c>
@@ -6794,8 +6182,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -6822,7 +6208,6 @@
       <c r="A39" t="n">
         <v>38</v>
       </c>
-      <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
           <t>SUTT Ujung Berung - Gedebage (arah sisi Bandung Selatan)</t>
@@ -6843,7 +6228,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
       <c r="H39" t="n">
         <v>2</v>
       </c>
@@ -6857,8 +6241,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -6885,7 +6267,6 @@
       <c r="A40" t="n">
         <v>39</v>
       </c>
-      <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
           <t>SUTT Ujung Berung - Bandung Timur</t>
@@ -6906,7 +6287,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
       <c r="H40" t="n">
         <v>2</v>
       </c>
@@ -6920,8 +6300,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -6948,7 +6326,6 @@
       <c r="A41" t="n">
         <v>40</v>
       </c>
-      <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
           <t>Outlet PLTA Parakan</t>
@@ -6969,7 +6346,6 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
       <c r="H41" t="n">
         <v>1</v>
       </c>
@@ -6983,8 +6359,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -7036,7 +6410,6 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
         <v>2</v>
       </c>
@@ -7050,8 +6423,6 @@
           <t>Sangat Rawan</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -7078,7 +6449,6 @@
       <c r="A43" t="n">
         <v>42</v>
       </c>
-      <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
           <t>SUTT 70 kV Parakan - Kadipaten</t>
@@ -7099,7 +6469,6 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
         <v>2</v>
       </c>
@@ -7113,8 +6482,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -7141,7 +6508,6 @@
       <c r="A44" t="n">
         <v>43</v>
       </c>
-      <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
           <t>SUTT 70 kV Sumedang - Kadipaten</t>
@@ -7162,7 +6528,6 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
         <v>2</v>
       </c>
@@ -7176,8 +6541,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -7204,7 +6567,6 @@
       <c r="A45" t="n">
         <v>44</v>
       </c>
-      <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
           <t>SUTT 70 kV Kadipaten - Arjawinangun (arah SS Mandirancan)</t>
@@ -7225,7 +6587,6 @@
           <t>70 kV</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
         <v>2</v>
       </c>
@@ -7239,8 +6600,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -7292,7 +6651,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
       <c r="H46" t="n">
         <v>2</v>
       </c>
@@ -7306,8 +6664,6 @@
           <t>Sangat Rawan</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -7334,7 +6690,6 @@
       <c r="A47" t="n">
         <v>46</v>
       </c>
-      <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
           <t>SUTT Ujung Berung - Traksi Tagolar</t>
@@ -7355,7 +6710,6 @@
           <t>150 kV</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
       <c r="H47" t="n">
         <v>1</v>
       </c>
@@ -7369,8 +6723,6 @@
           <t>Normal</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr">
         <is>
           <t>Jawa Barat</t>
@@ -7496,7 +6848,6 @@
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>NUBRG</t>
@@ -7540,7 +6891,6 @@
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>BDGSEL</t>
@@ -7584,7 +6934,6 @@
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>BDGSEL;NUBRG</t>
@@ -7628,7 +6977,6 @@
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>NUBRG</t>
@@ -7672,7 +7020,6 @@
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>BDGSEL;NUBRG</t>
@@ -7716,7 +7063,6 @@
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
           <t>BDGSEL</t>
@@ -7760,7 +7106,6 @@
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
           <t>BDGSEL</t>
@@ -7804,7 +7149,6 @@
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
           <t>NUBRG</t>
@@ -7848,7 +7192,6 @@
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
           <t>NUBRG</t>
@@ -7892,7 +7235,6 @@
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>BDGSEL</t>
@@ -7936,7 +7278,6 @@
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
           <t>BDGSEL;NUBRG</t>
@@ -7980,7 +7321,6 @@
           <t>Beroperasi</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
           <t>NUBRG</t>
@@ -8069,7 +7409,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Jangka Pendek: 1. Pembangunan GITET Cikalong (IBT dan outlet) Sesuai RUPTL 2025 - 2034, COD 2027. Jangka Menengah: 2. Pembangunan SUTT 150 kV Jawa Barat Landing Point (BDSLN-WYNDU-KMJNG- DRJAT). Sesuai RUPTL 2025- 2034, COD bertahap 2026 (BDSLN-WYNDU-KMJNG), 2027 (TSBRU-CAMIS) dan 2029-2030 (KMJNG-DRJAT)</t>
+          <t>Jangka Pendek: 1. Pembangunan GITET Cikalong (IBT dan outlet) Sesuai RUPTL 2025 - 2034, COD 2027. Jangka Menengah: 2. Pembangunan SUTT 150 kV Jawa Barat Landing Point (BDSLN-WYNDU-KMJNG- DRJAT). Sesuai RUPTL 2025 - 2034, COD bertahap 2026 (BDSLN-WYNDU-KMJNG), 2027 (TSBRU-CAMIS) dan 2029-2030 (KMJNG-DRJAT)</t>
         </is>
       </c>
     </row>
@@ -8104,7 +7444,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Jangka Pendek: Pembangunan SUTT 150 kV baru Bandung Selatan- Wayangwindu (Jawa Barat Landing Point) dengan kapasitas1600 A per sirkit. Sesuai RUPTL 2025-2034, COD 2026</t>
+          <t>Jangka Pendek: Pembangunan SUTT 150 kV baru Bandung Selatan- Wayangwindu (Jawa Barat Landing Point) dengan kapasitas1600 A per sirkit. Sesuai RUPTL 2025 -2034, COD 2026</t>
         </is>
       </c>
     </row>
@@ -8139,7 +7479,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Jangka Panjang: Pembangunan jalur baru SUTT 150 kV Cianjur-Padalarang Baru 1,2 (ByPass ke Subsistem Cirata) New 2cct, ACSR, 2xZebra, 1600 A, 83,2 kms. Proyek ini diperlukan guna mengantisipasi jika SUTT eksisting Cianjur-Rajamandala- Cigereleng trip 1 sirkit, maka terjadi Overload, Sesuai RUPTL 2025-2034, COD 2032</t>
+          <t>Jangka Panjang: Pembangunan jalur baru SUTT 150 kV Cianjur-Padalarang Baru 1,2 (ByPass ke Subsistem Cirata) New 2cct, ACSR, 2xZebra, 1600 A, 83,2 kms. Proyek ini diperlukan guna mengantisipasi jika SUTT eksisting Cianjur-Rajamandala- Cigereleng trip 1 sirkit, maka terjadi Overload, Sesuai RUPTL 2025 -2034, COD 2032</t>
         </is>
       </c>
     </row>
@@ -8194,7 +7534,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>[BELUM_DITETAPKAN] Kurang andalnya pasokan ke Traksi Tegalluar dikarenakan konfigurasi Traksi Tegalluar tapping di SUTT 150 kV Ujung Berung -Gedebage #1 #2</t>
+          <t>[BELUM_DITETAPKAN] Kurang andalnya pasokan ke Traksi Tegalluar dikarenakan konfigurasi Traksi Tegalluar tapping di SUTT 150 kV Ujung Berung - Gedebage #1 #2</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -8209,7 +7549,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Jangka Pendek : Pembangunan GIS Tegal Luar. Sesuai RUPTL 2025-2034, COD 2025 (Update COD Oktober 2026)</t>
+          <t>Jangka Pendek : Pembangunan GIS Tegal Luar. Sesuai RUPTL 2025 -2034, COD 2025 (Update COD Oktober 2026)</t>
         </is>
       </c>
     </row>
@@ -8349,7 +7689,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Jangka Pendek: 1. Pembangunan GITET Cikalong (IBT dan outlet) Sesuai RUPTL 2025 - 2034, COD 2027. Jangka Menengah: 2. Pembangunan SUTT 150 kV Jawa Barat Landing Point (BDSLN-WYNDU-KMJNG- DRJAT). Sesuai RUPTL 2025- 2034, COD bertahap 2026 (BDSLN-WYNDU-KMJNG), 2027 (TSBRU-CAMIS) dan 2029-2030 (KMJNG-DRJAT)</t>
+          <t>Jangka Pendek: 1. Pembangunan GITET Cikalong (IBT dan outlet) Sesuai RUPTL 2025 - 2034, COD 2027. Jangka Menengah: 2. Pembangunan SUTT 150 kV Jawa Barat Landing Point (BDSLN-WYNDU-KMJNG- DRJAT). Sesuai RUPTL 2025 - 2034, COD bertahap 2026 (BDSLN-WYNDU-KMJNG), 2027 (TSBRU-CAMIS) dan 2029-2030 (KMJNG-DRJAT)</t>
         </is>
       </c>
     </row>
@@ -8384,7 +7724,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Jangka Menengah: Rekonduktoring SUTT Kamojang-Darajat 1,2 menjadi 2cct, 2xZebra, 1600 A Sesuai RUPTL 2025-2034, COD 2029. Usulan sesuai dengan KKP Jawa Barat Landing Point, proyek ini dibutuhkan masuk di Tahun 2026</t>
+          <t>Jangka Menengah: Rekonduktoring SUTT Kamojang-Darajat 1,2 menjadi 2cct, 2xZebra, 1600 A Sesuai RUPTL 2025 -2034, COD 2029. Usulan sesuai dengan KKP Jawa Barat Landing Point, proyek ini dibutuhkan masuk di Tahun 2026</t>
         </is>
       </c>
     </row>
@@ -8414,7 +7754,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1. Pekerjaan tidak paralel dengan SUTT Sunyaragi-Jatigede- New Kadipaten</t>
+          <t>1. Pekerjaan tidak paralel dengan SUTT Sunyaragi -Jatigede- New Kadipaten</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -8454,7 +7794,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Jangka Pendek : Pembangunan GI 150 kV Sumedang Baru beserta outlet- nya. Sesuai RUPTL 2025-2034, COD 2027</t>
+          <t>Jangka Pendek : Pembangunan GI 150 kV Sumedang Baru beserta outlet- nya. Sesuai RUPTL 2025 -2034, COD 2027</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Offer a split subsystem on one sheet too (GABUNGAN view)
A subsystem split into regional views (Sumbagteng: Riau / Sumbar / Jambi)
could only be read panel by panel. A Views row keyed GABUNGAN now publishes
one more view holding every object and line of the subsystem, and every
view's sources when it names none. It is opt-in per workbook: tried on all
six split subsystems, it draws cleanly for Sumbagteng, Pelabuhan Ratu and
Bandung Selatan-Ujungberung (0 geometry findings, audit 42/42), which now
carry it; Cibatu 3,4-Mandirancan drops three lines as one sheet, Muarakarang-
Durikosambi finds no channel, and Sumbagut takes ~15 min to route.

The viewer shows a subsystem's views as a switcher on the drawing itself
("Sudut pandang: Riau | Sumatera Barat | Jambi | Gabungan"), keeps the
kerawanan in focus across the switch, and the tree marks the combined view
"semua dalam satu SLD".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/ss_bdgsel_nubrg_ingest.xlsx
+++ b/samples/ss_bdgsel_nubrg_ingest.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,6 +558,21 @@
         </is>
       </c>
       <c r="D3" t="n">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GABUNGAN</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Gabungan kedua sisi</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
         <v>127</v>
       </c>
     </row>

</xml_diff>